<commit_message>
feat: dokumentasi multi-foto (3-5) + video, TTD digital reuse, KOP PDF, slideshow, label Prodi, README lengkap
- laporan.html: foto sebelum/sesudah 3-5 + 1 video (maks 25MB), kompres foto otomatis
- TTD digital (canvas) + dropdown TTD tersimpan per prodi + peringatan & konfirmasi
- output PDF ber-KOP + unduh ulang (localStorage)
- index.html: slideshow dokumentasi foto + label Program Studi
- Code.gs: getTtd, simpan TTD & video ke Drive, getDashboard fotos (multi-URL)
- xlsx: data dummy + kolom Video + header Program Studi
- README: setup developer s/d cara pakai user
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_JumatBersih.xlsx
+++ b/Template_Spreadsheet_JumatBersih.xlsx
@@ -445,35 +445,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
-    <col width="26" customWidth="1" min="24" max="24"/>
-    <col width="26" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,7 +501,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Prodi</t>
+          <t>Program Studi</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -599,19 +601,29 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Foto Tambahan</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Waktu Kirim</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>TTD Ketua Jurusan</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>TTD Ka Prodi</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-12 09:42:00</t>
+          <t>2026-06-19 09.42:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -621,7 +633,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -646,89 +658,903 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>08123456789</t>
+          <t>6281234567801</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang kelas, Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Kotor</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Sangat Bersih</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Dr. Andi Wijaya, M.Kes</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>198001012005011001</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Ns. Budi Santoso, M.Kep</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>198501012010012001</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/kep_sb1/640/400, https://picsum.photos/seed/kep_sb2/640/400, https://picsum.photos/seed/kep_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/kep_ss1/640/400, https://picsum.photos/seed/kep_ss2/640/400, https://picsum.photos/seed/kep_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>09.42 WIB</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-19 10.15:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/002/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kebidanan</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bdn. Sri Lestari, M.Keb</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198607122011012002</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6281234567802</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
         <v>3</v>
       </c>
-      <c r="K2" t="n">
-        <v>9</v>
-      </c>
-      <c r="L2" t="n">
-        <v>17</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Pembersihan ruang kelas, Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang laboratorium, Penataan dokumen &amp; arsip</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Cukup Bersih</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Bersih</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Dr. Maya Sari, M.Kes</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>198102022006012001</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Bdn. Sri Lestari, M.Keb</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>198607122011012002</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/bid_sb1/640/400, https://picsum.photos/seed/bid_sb2/640/400, https://picsum.photos/seed/bid_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/bid_ss1/640/400, https://picsum.photos/seed/bid_ss2/640/400, https://picsum.photos/seed/bid_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>10.15 WIB</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-19 11.05:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/003/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gizi</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rina Marlina, M.Gizi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198803152012012003</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>6281234567803</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang dosen, Perawatan tanaman / penghijauan lingkungan</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>Kotor</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Bersih</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Dr. Hadi P, M.Kes</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>197905052004011002</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Rina Marlina, M.Gizi</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>198803152012012003</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/giz_sb1/640/400, https://picsum.photos/seed/giz_sb2/640/400, https://picsum.photos/seed/giz_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/giz_ss1/640/400, https://picsum.photos/seed/giz_ss2/640/400, https://picsum.photos/seed/giz_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>11.05 WIB</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-19 09.50:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/004/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sanitasi Lingkungan</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198409102010011004</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>6281234567804</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Gotong royong halaman / area parkir, Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Sangat Kotor</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>Sangat Bersih</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Perlu tambahan alat kebersihan</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Dr. Hadi P, M.Kes</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>197905052004011002</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>198409102010011004</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/san_sb1/640/400, https://picsum.photos/seed/san_sb2/640/400, https://picsum.photos/seed/san_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/san_ss1/640/400, https://picsum.photos/seed/san_ss2/640/400, https://picsum.photos/seed/san_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>09.50 WIB</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-19 11.20:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/005/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Analis Kesehatan / TLM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Dewi Anggraini, M.Si</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198711202013012005</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>6281234567805</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang laboratorium, Penataan meja &amp; kursi (Clean Desk Culture / 5R)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Cukup Bersih</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Sangat Bersih</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Dr. Maya Sari, M.Kes</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>198102022006012001</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Dewi Anggraini, M.Si</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>198711202013012005</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/tlm_sb1/640/400, https://picsum.photos/seed/tlm_sb2/640/400, https://picsum.photos/seed/tlm_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/tlm_ss1/640/400, https://picsum.photos/seed/tlm_ss2/640/400, https://picsum.photos/seed/tlm_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>11.20 WIB</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-19 10.33:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/006/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Farmasi</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Apt. Fajar Nugroho, M.Farm</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198512052011011006</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>6281234567806</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang arsip, Penataan dokumen &amp; arsip</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Kotor</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Bersih</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>Dr. Andi Wijaya, M.Kes</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>198001012005011001</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Ns. Budi Santoso, M.Kep</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>198501012010012001</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/...sebelum</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/...sesudah</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>09.42 WIB</t>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Apt. Fajar Nugroho, M.Farm</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>198512052011011006</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/far_sb1/640/400, https://picsum.photos/seed/far_sb2/640/400, https://picsum.photos/seed/far_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/far_ss1/640/400, https://picsum.photos/seed/far_ss2/640/400, https://picsum.photos/seed/far_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>10.33 WIB</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-19 08.55:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/007/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Teknik Elektromedik</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Yoga Pratama, M.T</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Kaprodi / 198902152014011007</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>6281234567807</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Pembersihan koridor dan area bersama, Pembersihan kamar mandi dan wastafel</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Kotor</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Cukup Bersih</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Dr. Hadi P, M.Kes</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>197905052004011002</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Yoga Pratama, M.T</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>198902152014011007</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/tem_sb1/640/400, https://picsum.photos/seed/tem_sb2/640/400, https://picsum.photos/seed/tem_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/tem_ss1/640/400, https://picsum.photos/seed/tem_ss2/640/400, https://picsum.photos/seed/tem_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>08.55 WIB</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -748,13 +1574,13 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Prodi / Jurusan</t>
+          <t>Program Studi</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -776,12 +1602,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567801</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.keperawatan@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -793,12 +1619,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567802</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.kebidanan@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -810,12 +1636,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567808</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.keperawatangigi@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -827,12 +1653,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567803</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.gizi@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -844,12 +1670,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567804</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.sanitasilingkungan@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -861,12 +1687,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567805</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.analiskesehatan@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -878,12 +1704,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567806</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.farmasi@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -895,12 +1721,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567809</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.rekammedis@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -912,12 +1738,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567810</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.fisioterapi@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
@@ -929,12 +1755,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>628xxxxxxxxxx</t>
+          <t>6281234567807</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kaprodi@poltekkespalembang.ac.id</t>
+          <t>kaprodi.teknikelektromedik@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
change: video via link (Drive/YouTube) ganti upload file; kompres foto 1280px/0.8
- hemat penyimpanan Drive institusi 100GB (video tak di-upload)
- foto auto-kompres lebih tajam (1280px, JPEG 0.8, ±300KB)
- Code.gs: simpan video sebagai link, bukan file
- README: penjelasan keterbatasan video + estimasi storage
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_JumatBersih.xlsx
+++ b/Template_Spreadsheet_JumatBersih.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://youtu.be/contoh-jumatbersih-keperawatan</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://drive.google.com/file/d/contoh123/view</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">

</xml_diff>

<commit_message>
feat: pratinjau 2-kolom, config dinamis di Sheet, URL relatif, penomoran anti-duplikat
- laporan.html: layout form + pratinjau PDF live (sebelahan di desktop, tumpuk di HP)
- Code.gs: tab Pengaturan (key-value) untuk variabel dinamis (NAMA_INSTANSI, EMAIL_ADMIN, BASE_URL, dll); _settings()/_formUrl()
- URL notifikasi dari BASE_URL (Sheet) + link frontend relatif (mudah pindah domain)
- penomoran pakai LockService + flush() agar tidak duplikat saat submit bersamaan
- xlsx: tambah tab Pengaturan; README diperbarui (lock, config sheet, relatif URL)
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_JumatBersih.xlsx
+++ b/Template_Spreadsheet_JumatBersih.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Laporan-JumatBersih" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Prodi-Master" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pengaturan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1767,4 +1768,159 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Kunci</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Nilai</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NAMA_INSTANSI</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Politeknik Kesehatan Kemenkes Palembang</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nama instansi di notifikasi &amp; PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EMAIL_ADMIN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>smartchampion@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Penerima rekap mingguan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BASE_URL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://smartchampion-jumatbersih.vercel.app</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Domain aplikasi — ubah saat pindah ke domain instansi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NOMOR_PREFIX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Prefix nomor laporan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BATAS_WAKTU</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15.00 WIB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Batas pengumpulan laporan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EMAIL_AKTIF</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Aktifkan notifikasi Email (TRUE/FALSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WA_AKTIF</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Aktifkan notifikasi WhatsApp (TRUE/FALSE)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: master Mengetahui & Penanggung Jawab + Aktivitas dataset, 11 unit jurusan/prodi, foto sebelum/sesudah dipisah, TTD lebih tebal
- daftar unit jadi 11 (campuran Jurusan dalam kota + PS/Prodi luar kota), label 'Jurusan / Program Studi'
- sheet Mengetahui (unit+kajur+kontak+TTD) → dropdown Mengetahui + sumber notifikasi
- sheet Penanggung Jawab (fleksibel, tumbuh otomatis) → dropdown PJ; pilih nama auto-isi NIP + TTD
- Aktivitas jadi dataset (tab Aktivitas), 'lainnya' auto-nambah ke dataset
- TTD dipakai ulang via link tersimpan (thumbnail Drive), _saveTtd pass-through link
- PDF: Foto Sebelum & Sesudah jadi 2 section terpisah (E & F), Pernyataan jadi G
- TTD: garis nama lebih tebal, modal proporsional (aspect 5/2), goresan pena lebih tebal
- xlsx: skema final 5 tab; README + kontrak API diperbarui
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_JumatBersih.xlsx
+++ b/Template_Spreadsheet_JumatBersih.xlsx
@@ -8,8 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Laporan-JumatBersih" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Prodi-Master" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pengaturan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mengetahui" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Penanggung Jawab" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Aktivitas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pengaturan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -73,13 +75,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -446,37 +445,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="30" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,7 +643,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Keperawatan</t>
+          <t>Jurusan Keperawatan</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -654,7 +653,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Kaprodi / 198501012010012001</t>
+          <t>Kajur / 198501012010012001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -676,7 +675,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Pembersihan ruang kelas, Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -706,12 +705,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Dr. Andi Wijaya, M.Kes</t>
+          <t>Ns. Budi Santoso, M.Kep</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>198001012005011001</t>
+          <t>198501012010012001</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -736,7 +735,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>https://youtu.be/contoh-jumatbersih-keperawatan</t>
+          <t>https://youtu.be/contoh-jb</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -778,12 +777,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Kebidanan</t>
+          <t>PS-Diploma Tiga Keperawatan Baturaja</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bdn. Sri Lestari, M.Keb</t>
+          <t>Ns. Lia Amelia, M.Kep</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -810,7 +809,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Pembersihan ruang laboratorium, Penataan dokumen &amp; arsip</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -820,12 +819,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Cukup Bersih</t>
+          <t>Kotor</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Bersih</t>
+          <t>Sangat Bersih</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -840,17 +839,17 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Dr. Maya Sari, M.Kes</t>
+          <t>Ns. Lia Amelia, M.Kep</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>198102022006012001</t>
+          <t>198607122011012002</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Bdn. Sri Lestari, M.Keb</t>
+          <t>Ns. Lia Amelia, M.Kep</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -860,17 +859,17 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/bid_sb1/640/400, https://picsum.photos/seed/bid_sb2/640/400, https://picsum.photos/seed/bid_sb3/640/400</t>
+          <t>https://picsum.photos/seed/btr_sb1/640/400, https://picsum.photos/seed/btr_sb2/640/400, https://picsum.photos/seed/btr_sb3/640/400</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/bid_ss1/640/400, https://picsum.photos/seed/bid_ss2/640/400, https://picsum.photos/seed/bid_ss3/640/400</t>
+          <t>https://picsum.photos/seed/btr_ss1/640/400, https://picsum.photos/seed/btr_ss2/640/400, https://picsum.photos/seed/btr_ss3/640/400</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/contoh123/view</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -912,12 +911,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Gizi</t>
+          <t>PS-Diploma Tiga Keperawatan Lahat</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rina Marlina, M.Gizi</t>
+          <t>Ns. Rahmat H, M.Kep</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -944,7 +943,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Pembersihan ruang dosen, Perawatan tanaman / penghijauan lingkungan</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -959,7 +958,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Bersih</t>
+          <t>Sangat Bersih</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -974,17 +973,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Dr. Hadi P, M.Kes</t>
+          <t>Ns. Rahmat H, M.Kep</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>197905052004011002</t>
+          <t>198803152012012003</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Rina Marlina, M.Gizi</t>
+          <t>Ns. Rahmat H, M.Kep</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -994,12 +993,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/giz_sb1/640/400, https://picsum.photos/seed/giz_sb2/640/400, https://picsum.photos/seed/giz_sb3/640/400</t>
+          <t>https://picsum.photos/seed/lht_sb1/640/400, https://picsum.photos/seed/lht_sb2/640/400, https://picsum.photos/seed/lht_sb3/640/400</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/giz_ss1/640/400, https://picsum.photos/seed/giz_ss2/640/400, https://picsum.photos/seed/giz_ss3/640/400</t>
+          <t>https://picsum.photos/seed/lht_ss1/640/400, https://picsum.photos/seed/lht_ss2/640/400, https://picsum.photos/seed/lht_ss3/640/400</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1046,17 +1045,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sanitasi Lingkungan</t>
+          <t>Jurusan Gizi</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Agus Salim, M.KL</t>
+          <t>Rina Marlina, M.Gizi</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Kaprodi / 198409102010011004</t>
+          <t>Kajur / 198409102010011004</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1078,7 +1077,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Gotong royong halaman / area parkir, Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1088,7 +1087,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Sangat Kotor</t>
+          <t>Kotor</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1108,17 +1107,17 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Dr. Hadi P, M.Kes</t>
+          <t>Rina Marlina, M.Gizi</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>197905052004011002</t>
+          <t>198409102010011004</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Agus Salim, M.KL</t>
+          <t>Rina Marlina, M.Gizi</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1128,12 +1127,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/san_sb1/640/400, https://picsum.photos/seed/san_sb2/640/400, https://picsum.photos/seed/san_sb3/640/400</t>
+          <t>https://picsum.photos/seed/giz_sb1/640/400, https://picsum.photos/seed/giz_sb2/640/400, https://picsum.photos/seed/giz_sb3/640/400</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/san_ss1/640/400, https://picsum.photos/seed/san_ss2/640/400, https://picsum.photos/seed/san_ss3/640/400</t>
+          <t>https://picsum.photos/seed/giz_ss1/640/400, https://picsum.photos/seed/giz_ss2/640/400, https://picsum.photos/seed/giz_ss3/640/400</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1180,17 +1179,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Analis Kesehatan / TLM</t>
+          <t>Jurusan Kebidanan</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Dewi Anggraini, M.Si</t>
+          <t>Bdn. Sri Lestari, M.Keb</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Kaprodi / 198711202013012005</t>
+          <t>Kajur / 198711202013012005</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1212,7 +1211,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Pembersihan ruang laboratorium, Penataan meja &amp; kursi (Clean Desk Culture / 5R)</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1222,7 +1221,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Cukup Bersih</t>
+          <t>Kotor</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1242,17 +1241,17 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Dr. Maya Sari, M.Kes</t>
+          <t>Bdn. Sri Lestari, M.Keb</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>198102022006012001</t>
+          <t>198711202013012005</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Dewi Anggraini, M.Si</t>
+          <t>Bdn. Sri Lestari, M.Keb</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1262,12 +1261,12 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/tlm_sb1/640/400, https://picsum.photos/seed/tlm_sb2/640/400, https://picsum.photos/seed/tlm_sb3/640/400</t>
+          <t>https://picsum.photos/seed/bid_sb1/640/400, https://picsum.photos/seed/bid_sb2/640/400, https://picsum.photos/seed/bid_sb3/640/400</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/tlm_ss1/640/400, https://picsum.photos/seed/tlm_ss2/640/400, https://picsum.photos/seed/tlm_ss3/640/400</t>
+          <t>https://picsum.photos/seed/bid_ss1/640/400, https://picsum.photos/seed/bid_ss2/640/400, https://picsum.photos/seed/bid_ss3/640/400</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1314,17 +1313,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Farmasi</t>
+          <t>Jurusan Farmasi</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Apt. Fajar Nugroho, M.Farm</t>
+          <t>Apt. Fajar N, M.Farm</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Kaprodi / 198512052011011006</t>
+          <t>Kajur / 198512052011011006</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1346,7 +1345,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Pembersihan ruang arsip, Penataan dokumen &amp; arsip</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1361,7 +1360,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Bersih</t>
+          <t>Sangat Bersih</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1376,17 +1375,17 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Dr. Andi Wijaya, M.Kes</t>
+          <t>Apt. Fajar N, M.Farm</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>198001012005011001</t>
+          <t>198512052011011006</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Apt. Fajar Nugroho, M.Farm</t>
+          <t>Apt. Fajar N, M.Farm</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1448,17 +1447,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Teknik Elektromedik</t>
+          <t>Jurusan Teknologi Laboratorium Medis</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Yoga Pratama, M.T</t>
+          <t>Dewi Anggraini, M.Si</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Kaprodi / 198902152014011007</t>
+          <t>Kajur / 198902152014011007</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1480,7 +1479,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Pembersihan koridor dan area bersama, Pembersihan kamar mandi dan wastafel</t>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1495,7 +1494,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Cukup Bersih</t>
+          <t>Sangat Bersih</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1510,17 +1509,17 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Dr. Hadi P, M.Kes</t>
+          <t>Dewi Anggraini, M.Si</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>197905052004011002</t>
+          <t>198902152014011007</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Yoga Pratama, M.T</t>
+          <t>Dewi Anggraini, M.Si</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1530,12 +1529,12 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/tem_sb1/640/400, https://picsum.photos/seed/tem_sb2/640/400, https://picsum.photos/seed/tem_sb3/640/400</t>
+          <t>https://picsum.photos/seed/tlm_sb1/640/400, https://picsum.photos/seed/tlm_sb2/640/400, https://picsum.photos/seed/tlm_sb3/640/400</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>https://picsum.photos/seed/tem_ss1/640/400, https://picsum.photos/seed/tem_ss2/640/400, https://picsum.photos/seed/tem_ss3/640/400</t>
+          <t>https://picsum.photos/seed/tlm_ss1/640/400, https://picsum.photos/seed/tlm_ss2/640/400, https://picsum.photos/seed/tlm_ss3/640/400</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1554,6 +1553,140 @@
         </is>
       </c>
       <c r="AB8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-19 10.05:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JB/SMART-CHAMPION/008/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Jumat</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Jurusan Kesehatan Lingkungan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Kajur / 198001012005011008</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>6281234567808</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang kelas, Pembersihan ruang laboratorium</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Kotor</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Sangat Bersih</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>198001012005011008</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>198001012005011008</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/ksl_sb1/640/400, https://picsum.photos/seed/ksl_sb2/640/400, https://picsum.photos/seed/ksl_sb3/640/400</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/seed/ksl_ss1/640/400, https://picsum.photos/seed/ksl_ss2/640/400, https://picsum.photos/seed/ksl_ss3/640/400</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>10.05 WIB</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1570,200 +1703,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Program Studi</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>No. WA (62...)</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Email Kaprodi/Kajur</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Jurusan/Prodi/Unit</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>No. HP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Email Jurusan/Prodi</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NIP</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TTD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Keperawatan</t>
+          <t>Jurusan Keperawatan</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Ns. Budi Santoso, M.Kep</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>6281234567801</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>kaprodi.keperawatan@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>keperawatan@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>198501012010012001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kebidanan</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+          <t>PS-Diploma Tiga Keperawatan Baturaja</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
         <is>
           <t>6281234567802</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>kaprodi.kebidanan@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>keperawatanbat@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Keperawatan Gigi</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>6281234567808</t>
-        </is>
-      </c>
+          <t>PS-Diploma Tiga Keperawatan Lubuklinggau</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kaprodi.keperawatangigi@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567803</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>keperawatanlub@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gizi</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>6281234567803</t>
-        </is>
-      </c>
+          <t>PS-Diploma Tiga Keperawatan Lahat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>kaprodi.gizi@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567804</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>keperawatanlah@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sanitasi Lingkungan</t>
+          <t>Jurusan Gizi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6281234567804</t>
+          <t>Rina Marlina, M.Gizi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>kaprodi.sanitasilingkungan@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567805</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gizi@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>198409102010011004</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Analis Kesehatan / TLM</t>
+          <t>Jurusan Kebidanan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6281234567805</t>
+          <t>Bdn. Sri Lestari, M.Keb</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>kaprodi.analiskesehatan@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567806</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>kebidanan@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>198711202013012005</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Farmasi</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>6281234567806</t>
-        </is>
-      </c>
+          <t>PS-Diploma Tiga Kebidanan Muara Enim</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kaprodi.farmasi@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567807</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>kebidananmuara@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Rekam Medis</t>
+          <t>Jurusan Farmasi</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6281234567809</t>
+          <t>Apt. Fajar N, M.Farm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kaprodi.rekammedis@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567808</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>farmasi@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>198512052011011006</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fisioterapi</t>
+          <t>Jurusan Teknologi Laboratorium Medis</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6281234567810</t>
+          <t>Dewi Anggraini, M.Si</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kaprodi.fisioterapi@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567809</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>teknologilabor@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>198902152014011007</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Teknik Elektromedik</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>6281234567807</t>
-        </is>
-      </c>
+          <t>Jurusan Kesehatan Gigi</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kaprodi.teknikelektromedik@poltekkespalembang.ac.id</t>
-        </is>
-      </c>
+          <t>6281234567810</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>kesehatangigi@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jurusan Kesehatan Lingkungan</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6281234567811</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kesehatanlingk@poltekkespalembang.ac.id</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>198001012005011008</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1776,26 +2025,334 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Jurusan/Prodi/Unit</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NIP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jurusan Keperawatan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ns. Budi Santoso, M.Kep</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>198501012010012001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PS-Diploma Tiga Keperawatan Baturaja</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ns. Lia Amelia, M.Kep</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>198607122011012002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PS-Diploma Tiga Keperawatan Lahat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ns. Rahmat H, M.Kep</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>198803152012012003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jurusan Gizi</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rina Marlina, M.Gizi</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>198409102010011004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jurusan Kebidanan</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bdn. Sri Lestari, M.Keb</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>198711202013012005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jurusan Farmasi</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Apt. Fajar N, M.Farm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>198512052011011006</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jurusan Teknologi Laboratorium Medis</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dewi Anggraini, M.Si</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>198902152014011007</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jurusan Kesehatan Lingkungan</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Agus Salim, M.KL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>198001012005011008</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Aktivitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang kelas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang laboratorium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang pimpinan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang administrasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang dosen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang arsip</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pembersihan ruang gudang</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pembersihan koridor dan area bersama</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Pembersihan kamar mandi dan wastafel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Pengelolaan sampah terpilah (organik &amp; anorganik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Penataan meja &amp; kursi (Clean Desk Culture / 5R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Penataan dokumen &amp; arsip</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Perawatan tanaman / penghijauan lingkungan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gotong royong halaman / area parkir</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Kunci</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nilai</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
@@ -1848,7 +2405,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Domain aplikasi — ubah saat pindah ke domain instansi</t>
+          <t>Domain aplikasi</t>
         </is>
       </c>
     </row>
@@ -1882,7 +2439,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Batas pengumpulan laporan</t>
+          <t>Batas (teks)</t>
         </is>
       </c>
     </row>
@@ -1899,7 +2456,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aktifkan notifikasi Email (TRUE/FALSE)</t>
+          <t>Notifikasi Email (TRUE/FALSE)</t>
         </is>
       </c>
     </row>
@@ -1916,7 +2473,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Aktifkan notifikasi WhatsApp (TRUE/FALSE)</t>
+          <t>Notifikasi WA (TRUE/FALSE)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: kolom laporan pakai Mengetahui/PJ + TTD tidak disimpan di baris laporan
- HEADERS: Nama Kajur/NIP Kajur/Nama Kaprodi/NIP Kaprodi -> Mengetahui/NIP Mengetahui/Penanggung Jawab/NIP PJ
- hapus kolom TTD Ketua Jurusan & TTD Ka Prodi dari sheet laporan (28->26 kolom)
- TTD melekat di sheet Mengetahui & Penanggung Jawab saja; gambar tersimpan sekali di Drive (link di master)
- _rowLaporan tidak lagi menulis TTD; ttd tetap disimpan ke master via _updateMengetahuiTtd/_simpanPJ
- xlsx: header laporan diperbarui (26 kolom, 96 baris dummy)
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_JumatBersih.xlsx
+++ b/Template_Spreadsheet_JumatBersih.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB97"/>
+  <dimension ref="A1:Z97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,26 +453,26 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
-    <col width="26" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
     <col width="11" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
@@ -571,22 +571,22 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Nama Kajur</t>
+          <t>Mengetahui</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>NIP Kajur</t>
+          <t>NIP Mengetahui</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Nama Kaprodi</t>
+          <t>Penanggung Jawab</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>NIP Kaprodi</t>
+          <t>NIP PJ</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -607,16 +607,6 @@
       <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Waktu Kirim</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>TTD Ketua Jurusan</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>TTD Ka Prodi</t>
         </is>
       </c>
     </row>
@@ -653,7 +643,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -743,12 +733,6 @@
           <t>09.02 WIB</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -783,7 +767,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000002</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -873,12 +857,6 @@
           <t>12.27 WIB</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -913,7 +891,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000003</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1003,12 +981,6 @@
           <t>09.02 WIB</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1043,7 +1015,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000004</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1133,12 +1105,6 @@
           <t>08.36 WIB</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1173,7 +1139,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000005</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1263,12 +1229,6 @@
           <t>12.45 WIB</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1303,7 +1263,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000006</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1393,12 +1353,6 @@
           <t>12.27 WIB</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1433,7 +1387,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000007</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1523,12 +1477,6 @@
           <t>10.46 WIB</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1563,7 +1511,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000008</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1653,12 +1601,6 @@
           <t>11.10 WIB</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1693,7 +1635,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000009</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1783,12 +1725,6 @@
           <t>08.48 WIB</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1823,7 +1759,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000010</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1913,12 +1849,6 @@
           <t>11.04 WIB</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1953,7 +1883,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000011</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2043,12 +1973,6 @@
           <t>10.41 WIB</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2083,7 +2007,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000012</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2173,12 +2097,6 @@
           <t>11.22 WIB</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2213,7 +2131,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000013</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2303,12 +2221,6 @@
           <t>11.25 WIB</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2343,7 +2255,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000014</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2433,12 +2345,6 @@
           <t>11.22 WIB</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2473,7 +2379,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000015</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2563,12 +2469,6 @@
           <t>09.42 WIB</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2603,7 +2503,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000016</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2693,12 +2593,6 @@
           <t>08.09 WIB</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2733,7 +2627,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000017</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2823,12 +2717,6 @@
           <t>12.39 WIB</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2863,7 +2751,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000018</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2953,12 +2841,6 @@
           <t>11.06 WIB</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2993,7 +2875,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000019</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3083,12 +2965,6 @@
           <t>11.10 WIB</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3123,7 +2999,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000020</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3213,12 +3089,6 @@
           <t>11.09 WIB</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3253,7 +3123,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000021</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -3343,12 +3213,6 @@
           <t>08.54 WIB</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3383,7 +3247,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000022</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -3473,12 +3337,6 @@
           <t>09.06 WIB</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3513,7 +3371,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000023</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3603,12 +3461,6 @@
           <t>09.33 WIB</t>
         </is>
       </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3643,7 +3495,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000024</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3733,12 +3585,6 @@
           <t>08.44 WIB</t>
         </is>
       </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3773,7 +3619,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000025</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3863,12 +3709,6 @@
           <t>12.49 WIB</t>
         </is>
       </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3903,7 +3743,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3993,12 +3833,6 @@
           <t>08.01 WIB</t>
         </is>
       </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4033,7 +3867,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000027</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4123,12 +3957,6 @@
           <t>10.23 WIB</t>
         </is>
       </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4163,7 +3991,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000028</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -4253,12 +4081,6 @@
           <t>10.13 WIB</t>
         </is>
       </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4293,7 +4115,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000029</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -4383,12 +4205,6 @@
           <t>08.58 WIB</t>
         </is>
       </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4423,7 +4239,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000030</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -4513,12 +4329,6 @@
           <t>10.05 WIB</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4553,7 +4363,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000031</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -4643,12 +4453,6 @@
           <t>09.01 WIB</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4683,7 +4487,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000032</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -4773,12 +4577,6 @@
           <t>12.35 WIB</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4813,7 +4611,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000033</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4903,12 +4701,6 @@
           <t>12.15 WIB</t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4943,7 +4735,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000034</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -5033,12 +4825,6 @@
           <t>10.57 WIB</t>
         </is>
       </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5073,7 +4859,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000035</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -5163,12 +4949,6 @@
           <t>12.32 WIB</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5203,7 +4983,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000036</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -5293,12 +5073,6 @@
           <t>09.30 WIB</t>
         </is>
       </c>
-      <c r="AA37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5333,7 +5107,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000037</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -5423,12 +5197,6 @@
           <t>12.33 WIB</t>
         </is>
       </c>
-      <c r="AA38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5463,7 +5231,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000038</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -5553,12 +5321,6 @@
           <t>10.02 WIB</t>
         </is>
       </c>
-      <c r="AA39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5593,7 +5355,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000039</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -5683,12 +5445,6 @@
           <t>10.39 WIB</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5723,7 +5479,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000040</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -5813,12 +5569,6 @@
           <t>08.25 WIB</t>
         </is>
       </c>
-      <c r="AA41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5853,7 +5603,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000041</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -5943,12 +5693,6 @@
           <t>09.42 WIB</t>
         </is>
       </c>
-      <c r="AA42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5983,7 +5727,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000042</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -6073,12 +5817,6 @@
           <t>09.29 WIB</t>
         </is>
       </c>
-      <c r="AA43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6113,7 +5851,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000043</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -6203,12 +5941,6 @@
           <t>09.10 WIB</t>
         </is>
       </c>
-      <c r="AA44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6243,7 +5975,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000044</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -6333,12 +6065,6 @@
           <t>10.05 WIB</t>
         </is>
       </c>
-      <c r="AA45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6373,7 +6099,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000045</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -6463,12 +6189,6 @@
           <t>08.24 WIB</t>
         </is>
       </c>
-      <c r="AA46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6503,7 +6223,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000046</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -6593,12 +6313,6 @@
           <t>08.05 WIB</t>
         </is>
       </c>
-      <c r="AA47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6633,7 +6347,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000047</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -6723,12 +6437,6 @@
           <t>11.54 WIB</t>
         </is>
       </c>
-      <c r="AA48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6763,7 +6471,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000048</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -6853,12 +6561,6 @@
           <t>10.03 WIB</t>
         </is>
       </c>
-      <c r="AA49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6893,7 +6595,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000049</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -6983,12 +6685,6 @@
           <t>10.35 WIB</t>
         </is>
       </c>
-      <c r="AA50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7023,7 +6719,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000050</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -7113,12 +6809,6 @@
           <t>09.07 WIB</t>
         </is>
       </c>
-      <c r="AA51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7153,7 +6843,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000051</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -7243,12 +6933,6 @@
           <t>10.33 WIB</t>
         </is>
       </c>
-      <c r="AA52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7283,7 +6967,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000052</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -7373,12 +7057,6 @@
           <t>08.16 WIB</t>
         </is>
       </c>
-      <c r="AA53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7413,7 +7091,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000053</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -7503,12 +7181,6 @@
           <t>09.59 WIB</t>
         </is>
       </c>
-      <c r="AA54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7543,7 +7215,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000054</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -7633,12 +7305,6 @@
           <t>12.19 WIB</t>
         </is>
       </c>
-      <c r="AA55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7673,7 +7339,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000055</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -7763,12 +7429,6 @@
           <t>10.03 WIB</t>
         </is>
       </c>
-      <c r="AA56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7803,7 +7463,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000056</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -7893,12 +7553,6 @@
           <t>08.05 WIB</t>
         </is>
       </c>
-      <c r="AA57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7933,7 +7587,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000057</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -8023,12 +7677,6 @@
           <t>09.02 WIB</t>
         </is>
       </c>
-      <c r="AA58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8063,7 +7711,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000058</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -8153,12 +7801,6 @@
           <t>11.05 WIB</t>
         </is>
       </c>
-      <c r="AA59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8193,7 +7835,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000059</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -8283,12 +7925,6 @@
           <t>08.05 WIB</t>
         </is>
       </c>
-      <c r="AA60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8323,7 +7959,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000060</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -8413,12 +8049,6 @@
           <t>08.19 WIB</t>
         </is>
       </c>
-      <c r="AA61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8453,7 +8083,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000061</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -8543,12 +8173,6 @@
           <t>11.09 WIB</t>
         </is>
       </c>
-      <c r="AA62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8583,7 +8207,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000062</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -8673,12 +8297,6 @@
           <t>12.48 WIB</t>
         </is>
       </c>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8713,7 +8331,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000063</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -8803,12 +8421,6 @@
           <t>08.08 WIB</t>
         </is>
       </c>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8843,7 +8455,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000064</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -8933,12 +8545,6 @@
           <t>08.40 WIB</t>
         </is>
       </c>
-      <c r="AA65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8973,7 +8579,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000065</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -9063,12 +8669,6 @@
           <t>08.47 WIB</t>
         </is>
       </c>
-      <c r="AA66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9103,7 +8703,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000066</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -9193,12 +8793,6 @@
           <t>11.58 WIB</t>
         </is>
       </c>
-      <c r="AA67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9233,7 +8827,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000067</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -9323,12 +8917,6 @@
           <t>09.21 WIB</t>
         </is>
       </c>
-      <c r="AA68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9363,7 +8951,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000068</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -9453,12 +9041,6 @@
           <t>08.31 WIB</t>
         </is>
       </c>
-      <c r="AA69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9493,7 +9075,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000069</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -9583,12 +9165,6 @@
           <t>12.18 WIB</t>
         </is>
       </c>
-      <c r="AA70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9623,7 +9199,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000070</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -9713,12 +9289,6 @@
           <t>10.05 WIB</t>
         </is>
       </c>
-      <c r="AA71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9753,7 +9323,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000071</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -9843,12 +9413,6 @@
           <t>11.17 WIB</t>
         </is>
       </c>
-      <c r="AA72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9883,7 +9447,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000072</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -9973,12 +9537,6 @@
           <t>12.16 WIB</t>
         </is>
       </c>
-      <c r="AA73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10013,7 +9571,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000073</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -10103,12 +9661,6 @@
           <t>10.14 WIB</t>
         </is>
       </c>
-      <c r="AA74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10143,7 +9695,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000074</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -10233,12 +9785,6 @@
           <t>11.43 WIB</t>
         </is>
       </c>
-      <c r="AA75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10273,7 +9819,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000075</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -10363,12 +9909,6 @@
           <t>10.16 WIB</t>
         </is>
       </c>
-      <c r="AA76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10403,7 +9943,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000076</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -10493,12 +10033,6 @@
           <t>11.48 WIB</t>
         </is>
       </c>
-      <c r="AA77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10533,7 +10067,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000077</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -10623,12 +10157,6 @@
           <t>10.40 WIB</t>
         </is>
       </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10663,7 +10191,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000078</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -10753,12 +10281,6 @@
           <t>09.49 WIB</t>
         </is>
       </c>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10793,7 +10315,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000079</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -10883,12 +10405,6 @@
           <t>09.46 WIB</t>
         </is>
       </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10923,7 +10439,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000080</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -11013,12 +10529,6 @@
           <t>10.31 WIB</t>
         </is>
       </c>
-      <c r="AA81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -11053,7 +10563,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000081</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -11143,12 +10653,6 @@
           <t>10.19 WIB</t>
         </is>
       </c>
-      <c r="AA82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -11183,7 +10687,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000082</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -11273,12 +10777,6 @@
           <t>12.42 WIB</t>
         </is>
       </c>
-      <c r="AA83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -11313,7 +10811,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000083</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -11403,12 +10901,6 @@
           <t>12.57 WIB</t>
         </is>
       </c>
-      <c r="AA84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -11443,7 +10935,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000084</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -11533,12 +11025,6 @@
           <t>09.35 WIB</t>
         </is>
       </c>
-      <c r="AA85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -11573,7 +11059,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000085</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -11663,12 +11149,6 @@
           <t>08.20 WIB</t>
         </is>
       </c>
-      <c r="AA86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11703,7 +11183,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000086</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -11793,12 +11273,6 @@
           <t>10.08 WIB</t>
         </is>
       </c>
-      <c r="AA87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -11833,7 +11307,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000087</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -11923,12 +11397,6 @@
           <t>11.41 WIB</t>
         </is>
       </c>
-      <c r="AA88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11963,7 +11431,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000088</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -12053,12 +11521,6 @@
           <t>11.45 WIB</t>
         </is>
       </c>
-      <c r="AA89" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -12093,7 +11555,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000089</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -12183,12 +11645,6 @@
           <t>11.28 WIB</t>
         </is>
       </c>
-      <c r="AA90" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -12223,7 +11679,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000090</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -12313,12 +11769,6 @@
           <t>08.52 WIB</t>
         </is>
       </c>
-      <c r="AA91" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -12353,7 +11803,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000091</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -12443,12 +11893,6 @@
           <t>09.36 WIB</t>
         </is>
       </c>
-      <c r="AA92" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -12483,7 +11927,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000092</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -12573,12 +12017,6 @@
           <t>11.44 WIB</t>
         </is>
       </c>
-      <c r="AA93" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12613,7 +12051,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000093</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -12703,12 +12141,6 @@
           <t>09.24 WIB</t>
         </is>
       </c>
-      <c r="AA94" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -12743,7 +12175,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000094</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -12833,12 +12265,6 @@
           <t>10.29 WIB</t>
         </is>
       </c>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -12873,7 +12299,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000095</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -12963,12 +12389,6 @@
           <t>12.15 WIB</t>
         </is>
       </c>
-      <c r="AA96" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13003,7 +12423,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Pelaksana / 1990xxxx</t>
+          <t>Pelaksana / 19900000096</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -13093,12 +12513,6 @@
           <t>11.56 WIB</t>
         </is>
       </c>
-      <c r="AA97" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB97" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>